<commit_message>
Fix study period, H2.2 result and assumptions note in chi-square workbook
</commit_message>
<xml_diff>
--- a/excel/chi_square_tests.xlsx
+++ b/excel/chi_square_tests.xlsx
@@ -60,7 +60,7 @@
     <t>Healthcare Appointment No-Show Analysis · Chi-Square Tests</t>
   </si>
   <si>
-    <t>Statistical tests behind the hypothesis tree · Medical Appointment No-Shows (Kaggle) · Vitória, Brazil · April–June 2016</t>
+    <t>Statistical tests behind the hypothesis tree · Medical Appointment No-Shows (Kaggle) · Vitória, Brazil · April 29 – June 8, 2016</t>
   </si>
   <si>
     <t>Valid appointments</t>
@@ -240,10 +240,10 @@
     <t>Lead-time group, SMS, age group, neighborhood... One test covers all groups at once.</t>
   </si>
   <si>
-    <t>Assumptions met</t>
-  </si>
-  <si>
-    <t>Independent observations and expected count ≥ 5 per cell. Small groups were excluded (Saturday, neighborhoods &lt; 200 appointments).</t>
+    <t>Assumptions</t>
+  </si>
+  <si>
+    <t>Expected count ≥ 5 per cell. Small groups were excluded (Saturday, neighborhoods &lt; 200 appointments). Some patients have several appointments, so observations are not fully independent.</t>
   </si>
   <si>
     <t>Transparent</t>
@@ -342,7 +342,7 @@
     <t>Period</t>
   </si>
   <si>
-    <t>April to June 2016 only; no-show history is truncated at the start of the period.</t>
+    <t>April 29 to June 8, 2016 only (about six weeks); no-show history is truncated at the start of the period.</t>
   </si>
   <si>
     <t>Colour legend</t>
@@ -735,7 +735,7 @@
     <t>Prior no-show</t>
   </si>
   <si>
-    <t>Patients with a prior no-show miss 26.9% of the time, 8.0 p.p. more than returning patients who never missed. About 87% of χ² comes from this group. First-time patients (19.4%) look like those who never missed. History only covers April–June 2016.</t>
+    <t>Patients with a prior no-show miss 26.9% of the time, 8.0 p.p. more than returning patients who never missed. About 87% of χ² comes from this group. First-time patients (19.4%) look like those who never missed. History only covers April 29 – June 8, 2016.</t>
   </si>
   <si>
     <t>H4.1 · Neighborhoods above average</t>
@@ -1790,9 +1790,10 @@
       <c r="C17" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="14" t="str">
-        <f>TEXT(MAX('H2.2_SMS_Controlled'!H9:H12),"0.0")&amp;" to "&amp;TEXT(MIN('H2.2_SMS_Controlled'!H9:H12),"0.0")&amp;" p.p. in groups of 4+ days"</f>
-        <v>-03 to -07 p.p. in groups of 4+ days</v>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>−3.1 to −7.3 p.p. in groups of 4+ days</t>
+        </is>
       </c>
       <c r="E17" s="16" t="str">
         <f>'H2.2_SMS_Controlled'!B20</f>

</xml_diff>